<commit_message>
Initial update for new latch memory structure...
</commit_message>
<xml_diff>
--- a/eFPGA Memory Sizes.xlsx
+++ b/eFPGA Memory Sizes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13561f3231cadc0a/DTU/Comp_Arch_2/eFPGA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="120" documentId="8_{5CDDF4ED-CFF6-4896-8902-F3B11B76877A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3EB51DCD-E65F-40DA-8C69-BC7837FF5D72}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{5CDDF4ED-CFF6-4896-8902-F3B11B76877A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E219349-8219-4352-A98D-FDC4602AB558}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{55F2CDF7-820B-407F-947D-0D6AA8888A49}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{55F2CDF7-820B-407F-947D-0D6AA8888A49}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -490,12 +490,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE99E594-1A45-4FC9-9FEB-756CEE2DE8B7}">
   <dimension ref="B2:R19"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
@@ -518,15 +518,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C3">
-        <v>2656</v>
+        <v>2848</v>
       </c>
       <c r="D3">
-        <v>2176</v>
+        <v>1728</v>
       </c>
       <c r="E3">
         <v>2352</v>
@@ -551,17 +551,17 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>7</v>
       </c>
       <c r="C4">
         <f>C3/32</f>
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D4">
         <f>D3/32</f>
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E4">
         <f>E3/32</f>
@@ -572,16 +572,16 @@
         <v>75</v>
       </c>
       <c r="I4">
-        <f>8*8</f>
-        <v>64</v>
+        <f>6*8</f>
+        <v>48</v>
       </c>
       <c r="J4">
-        <f>8*16</f>
-        <v>128</v>
+        <f>6*16</f>
+        <v>96</v>
       </c>
       <c r="L4">
-        <f>8*32</f>
-        <v>256</v>
+        <f>6*32</f>
+        <v>192</v>
       </c>
       <c r="P4">
         <f>16*2</f>
@@ -591,13 +591,13 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>8</v>
       </c>
       <c r="C5" s="3">
         <f>C4+D4</f>
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3">
@@ -619,25 +619,25 @@
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:18" x14ac:dyDescent="0.3">
       <c r="I6">
-        <f>8*8</f>
-        <v>64</v>
+        <f>6*8</f>
+        <v>48</v>
       </c>
       <c r="J6">
-        <f>8*16</f>
-        <v>128</v>
+        <f>6*16</f>
+        <v>96</v>
       </c>
       <c r="L6">
-        <f>8*32</f>
-        <v>256</v>
+        <f>6*32</f>
+        <v>192</v>
       </c>
       <c r="P6">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>9</v>
       </c>
@@ -656,17 +656,17 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>11</v>
       </c>
       <c r="C8">
         <f>C4</f>
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="D8">
         <f>D4</f>
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E8">
         <f>E4+E7/32</f>
@@ -677,25 +677,25 @@
         <v>75</v>
       </c>
       <c r="I8">
-        <f>8*8</f>
-        <v>64</v>
+        <f>6*8</f>
+        <v>48</v>
       </c>
       <c r="J8">
-        <f>8*16</f>
-        <v>128</v>
+        <f>6*16</f>
+        <v>96</v>
       </c>
       <c r="L8">
-        <f>8*32</f>
-        <v>256</v>
-      </c>
-    </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.35">
+        <f>6*32</f>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="9" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="3">
         <f>C8+D8</f>
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3">
@@ -710,21 +710,21 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:18" x14ac:dyDescent="0.3">
       <c r="I10">
-        <f>8*8</f>
-        <v>64</v>
+        <f>6*8</f>
+        <v>48</v>
       </c>
       <c r="J10">
-        <f>8*16</f>
-        <v>128</v>
+        <f>6*16</f>
+        <v>96</v>
       </c>
       <c r="L10">
-        <f>8*32</f>
-        <v>256</v>
-      </c>
-    </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.35">
+        <f>6*32</f>
+        <v>192</v>
+      </c>
+    </row>
+    <row r="11" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>13</v>
       </c>
@@ -733,26 +733,26 @@
         <v>224</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>14</v>
       </c>
       <c r="D12">
         <f>D8+D11/32</f>
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="F12">
         <f>F8</f>
         <v>75</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:18" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>18</v>
       </c>
       <c r="C13" s="3">
         <f>C9*2+D12</f>
-        <v>377</v>
+        <v>347</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="3">
@@ -768,7 +768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:18" x14ac:dyDescent="0.3">
       <c r="E15" s="1" t="s">
         <v>2</v>
       </c>
@@ -776,7 +776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:18" x14ac:dyDescent="0.3">
       <c r="C16">
         <f>32*6</f>
         <v>192</v>
@@ -814,7 +814,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="17" spans="3:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C17">
         <v>6</v>
       </c>
@@ -841,7 +841,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="18" spans="3:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="3:12" x14ac:dyDescent="0.3">
       <c r="C18">
         <f>16*6</f>
         <v>96</v>
@@ -878,14 +878,14 @@
         <v>512</v>
       </c>
     </row>
-    <row r="19" spans="3:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="3:12" x14ac:dyDescent="0.3">
       <c r="D19">
-        <f>10*4</f>
-        <v>40</v>
+        <f>10*6</f>
+        <v>60</v>
       </c>
       <c r="F19">
-        <f>10*4</f>
-        <v>40</v>
+        <f>10*6</f>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>